<commit_message>
Actualizar entregables del Sprint 2: responsables planificados y decisiones
- Responsables planificados por módulo en backlog y plan de pruebas.
- RR-09: despliegue local/pruebas para el MVP, nube en fase posterior.
- UC-13 (cliente internacional) definido como fuera del MVP.
- Notas de la demo y estado actual alineados con el prototipo de frontend.
- Se mantienen como [COMPLETAR] la autoría del Sprint 1, las contribuciones
  individuales y los resultados de las pruebas.
</commit_message>
<xml_diff>
--- a/docs/sprint2/Plan_de_Pruebas_CoffeeExport_Manager.xlsx
+++ b/docs/sprint2/Plan_de_Pruebas_CoffeeExport_Manager.xlsx
@@ -553,7 +553,7 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>[COMPLETAR] (propuesta: Brayan Guerrero)</t>
+          <t>Brayan Guerrero</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
@@ -607,7 +607,7 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>[COMPLETAR] (propuesta: Mario Zambrano)</t>
+          <t>Mario Zambrano</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
@@ -661,7 +661,7 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>[COMPLETAR] (propuesta: Brayan Guerrero)</t>
+          <t>Brayan Guerrero</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
@@ -715,7 +715,7 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>[COMPLETAR] (propuesta: Brayan Guerrero)</t>
+          <t>Brayan Guerrero</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
@@ -769,7 +769,7 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>[COMPLETAR] (propuesta: Juan Jurado)</t>
+          <t>Juan Jurado</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
@@ -823,7 +823,7 @@
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>[COMPLETAR] (propuesta: Juan Jurado)</t>
+          <t>Juan Jurado</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
@@ -877,7 +877,7 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>[COMPLETAR] (propuesta: Juan Jurado)</t>
+          <t>Juan Jurado</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
@@ -931,7 +931,7 @@
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>[COMPLETAR] (propuesta: Juan Jurado)</t>
+          <t>Juan Jurado</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
@@ -985,7 +985,7 @@
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>[COMPLETAR] (propuesta: Nicoll López)</t>
+          <t>Nicoll López</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
@@ -1039,7 +1039,7 @@
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>[COMPLETAR] (propuesta: Nicoll López)</t>
+          <t>Nicoll López</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
@@ -1093,7 +1093,7 @@
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>[COMPLETAR] (propuesta: Nicoll López)</t>
+          <t>Nicoll López</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
@@ -1147,7 +1147,7 @@
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>[COMPLETAR] (propuesta: Alexander Rodríguez)</t>
+          <t>Alexander Rodríguez</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
@@ -1201,7 +1201,7 @@
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>[COMPLETAR] (propuesta: Alexander Rodríguez)</t>
+          <t>Alexander Rodríguez</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
@@ -1255,7 +1255,7 @@
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>[COMPLETAR] (propuesta: Alexander Rodríguez)</t>
+          <t>Alexander Rodríguez</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
@@ -1309,7 +1309,7 @@
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>[COMPLETAR] (propuesta: Alexander Rodríguez)</t>
+          <t>Alexander Rodríguez</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
@@ -1363,7 +1363,7 @@
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>[COMPLETAR] (propuesta: Alexander Rodríguez)</t>
+          <t>Alexander Rodríguez</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
@@ -1417,7 +1417,7 @@
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>[COMPLETAR] (propuesta: Juan Jurado)</t>
+          <t>Juan Jurado</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
@@ -1471,7 +1471,7 @@
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>[COMPLETAR] (propuesta: Mario Zambrano)</t>
+          <t>Mario Zambrano</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
@@ -1525,7 +1525,7 @@
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>[COMPLETAR] (propuesta: Brayan Guerrero)</t>
+          <t>Brayan Guerrero</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
@@ -1579,7 +1579,7 @@
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>[COMPLETAR] (propuesta: Brayan Guerrero)</t>
+          <t>Brayan Guerrero</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
@@ -1633,7 +1633,7 @@
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>[COMPLETAR] (propuesta: Juan Jurado)</t>
+          <t>Juan Jurado</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
@@ -1687,7 +1687,7 @@
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>[COMPLETAR] (propuesta: Juan Jurado)</t>
+          <t>Juan Jurado</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
@@ -1741,7 +1741,7 @@
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>[COMPLETAR] (propuesta: Juan Jurado)</t>
+          <t>Juan Jurado</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
@@ -1795,7 +1795,7 @@
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>[COMPLETAR] (propuesta: Nicoll López)</t>
+          <t>Nicoll López</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
@@ -1849,7 +1849,7 @@
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>[COMPLETAR] (propuesta: Nicoll López)</t>
+          <t>Nicoll López</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
@@ -1903,7 +1903,7 @@
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>[COMPLETAR] (propuesta: Alexander Rodríguez)</t>
+          <t>Alexander Rodríguez</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
@@ -1957,7 +1957,7 @@
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>[COMPLETAR] (propuesta: Alexander Rodríguez)</t>
+          <t>Alexander Rodríguez</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
@@ -2011,7 +2011,7 @@
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>[COMPLETAR] (propuesta: Mario Zambrano)</t>
+          <t>Mario Zambrano</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
@@ -2065,7 +2065,7 @@
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>[COMPLETAR] (propuesta: Mario Zambrano)</t>
+          <t>Mario Zambrano</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
@@ -2119,7 +2119,7 @@
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>[COMPLETAR] (propuesta: Mario Zambrano)</t>
+          <t>Mario Zambrano</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
@@ -2173,7 +2173,7 @@
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>[COMPLETAR] (propuesta: Mario Zambrano)</t>
+          <t>Mario Zambrano</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
@@ -2227,7 +2227,7 @@
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>[COMPLETAR] (propuesta: Mario Zambrano)</t>
+          <t>Mario Zambrano</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
@@ -2281,7 +2281,7 @@
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>[COMPLETAR] (propuesta: Brayan Guerrero)</t>
+          <t>Brayan Guerrero</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
@@ -2335,7 +2335,7 @@
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>[COMPLETAR] (propuesta: Juan Jurado)</t>
+          <t>Juan Jurado</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
@@ -2389,7 +2389,7 @@
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>[COMPLETAR] (propuesta: Nicoll López)</t>
+          <t>Nicoll López</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
@@ -2443,7 +2443,7 @@
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>[COMPLETAR] (propuesta: Alexander Rodríguez)</t>
+          <t>Alexander Rodríguez</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
@@ -2497,7 +2497,7 @@
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>[COMPLETAR] (propuesta: Brayan Guerrero)</t>
+          <t>Brayan Guerrero</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
@@ -2551,7 +2551,7 @@
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>[COMPLETAR] (propuesta: Juan Jurado)</t>
+          <t>Juan Jurado</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
@@ -2605,7 +2605,7 @@
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>[COMPLETAR] (propuesta: Alexander Rodríguez)</t>
+          <t>Alexander Rodríguez</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
@@ -2659,7 +2659,7 @@
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>[COMPLETAR] (propuesta: Alexander Rodríguez)</t>
+          <t>Alexander Rodríguez</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
@@ -2713,7 +2713,7 @@
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>[COMPLETAR] (propuesta: Nicoll López)</t>
+          <t>Nicoll López</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
@@ -2767,7 +2767,7 @@
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>[COMPLETAR] (propuesta: Juan Jurado)</t>
+          <t>Juan Jurado</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
@@ -2821,7 +2821,7 @@
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>[COMPLETAR] (propuesta: Mario Zambrano)</t>
+          <t>Mario Zambrano</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
@@ -2875,7 +2875,7 @@
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>[COMPLETAR] (propuesta: Brayan Guerrero)</t>
+          <t>Brayan Guerrero</t>
         </is>
       </c>
       <c r="D50" s="3" t="inlineStr">

</xml_diff>